<commit_message>
fix(decks): answer the review of the fall week 2 deck
The AI demo now shows ephira's day-one map after the tool output, from one
map constant shared with the worked example. The reveal slide states what
the repository supports: the first version marked for the app store
(1.1.0) and what came later, with pregnancy mode as a later, separate mode.
The pipeline and research kickers read "a sketch from the project page",
and the notes drop first-person plural, the unsourced adopter claim, the
dated listing count, and the restated quality-bar line. The backbone slide
gives its reason, and the template URL comes from Astro.site.

The wrap slide and the template's Story map tab say to export the whole
workbook, both tabs, as one PDF. The fall Workshop 1 submission names the
minimum of four backbone columns and one complete walking-skeleton row and
says "research chain", and the activity intro drops epics.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/story-map-template.xlsx
+++ b/public/story-map-template.xlsx
@@ -31,7 +31,7 @@
     <t>Why, in one line</t>
   </si>
   <si>
-    <t>Start a story with ? when it is assumed, not yet checked with your partner: the cell turns amber, and the question goes on the Questions for our partner tab. A story without ? is known.</t>
+    <t>Start a story with ? when it is assumed, not yet checked with your partner: the cell turns amber, and the question goes on the Questions for our partner tab. A story without ? is known. To submit, export the whole workbook, both tabs, as one PDF (in Google Sheets, choose Workbook, not Current sheet).</t>
   </si>
   <si>
     <r>
@@ -714,7 +714,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
feat(assignments): define release rows and the one-map rule for several users
A map has as many release rows as a team needs: the walking skeleton is
the fall's, Release 1 the first iteration after it, later releases
follow, and Out of scope this year is the last row; a story's row marks
its scope. State it once on the Workshop 1 entry and relabel the
template's Release 1 row to match, with a note to insert more release
rows. A project with more than one kind of user draws one map, the
primary user's flow with parallel columns only where another path
diverges: one sentence on the activity, one note in the template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/story-map-template.xlsx
+++ b/public/story-map-template.xlsx
@@ -31,7 +31,7 @@
     <t>Why, in one line</t>
   </si>
   <si>
-    <t>Start a story with ? when it is assumed, not yet checked with your partner: the cell turns amber, and the question goes on the Questions for our partner tab. A story without ? is known. To submit, export the whole workbook, both tabs, as one PDF (in Google Sheets, choose Workbook, not Current sheet).</t>
+    <t>Start a story with ? when it is assumed, not yet checked with your partner: the cell turns amber, and the question goes on the Questions for our partner tab. A story without ? is known. Insert a row for each release after Release 1 (Release 2, Release 3), above Out of scope this year. More than one kind of user? Draw one map: follow the primary user's flow, and add parallel columns only where another user's path diverges. To submit, export the whole workbook, both tabs, as one PDF (in Google Sheets, choose Workbook, not Current sheet).</t>
   </si>
   <si>
     <r>
@@ -72,7 +72,7 @@
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">
-One story under every column, however thin.</t>
+One story under every column, however thin. Built in the fall.</t>
     </r>
   </si>
   <si>
@@ -93,7 +93,7 @@
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">
-The next slice.</t>
+The first iteration after the walking skeleton. Insert more release rows below it as needed.</t>
     </r>
   </si>
   <si>
@@ -714,7 +714,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>

</xml_diff>